<commit_message>
attendance percentage calculated and stored
</commit_message>
<xml_diff>
--- a/data/atten.xlsx
+++ b/data/atten.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="31">
   <si>
-    <t>reg no</t>
+    <t>register_number</t>
   </si>
   <si>
     <t>MON</t>
@@ -40,7 +40,7 @@
     <t>SUN</t>
   </si>
   <si>
-    <t>Phone No</t>
+    <t>phone_number</t>
   </si>
   <si>
     <t>927623bcs001</t>
@@ -124,7 +124,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -156,16 +156,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -481,18 +478,18 @@
   <dimension ref="A1:I21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="5" width="12.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="5" width="10.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="5" width="10.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="5" width="10.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="5" width="11.005" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="5" width="10.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="5" width="10.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="5" width="10.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="6" width="23.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="4" width="12.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="4" width="10.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="4" width="10.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="4" width="10.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="4" width="11.005" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="4" width="10.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="4" width="10.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="4" width="10.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="5" width="23.719285714285714" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -521,7 +518,7 @@
         <v>8</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="1" t="s">
         <v>9</v>
       </c>
@@ -546,11 +543,11 @@
       <c r="H2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="I2" s="4">
-        <v>6383592840</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+      <c r="I2" s="3">
+        <v>6383592840</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
@@ -575,11 +572,11 @@
       <c r="H3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="I3" s="4">
-        <v>6383592840</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+      <c r="I3" s="3">
+        <v>6383592840</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="1" t="s">
         <v>13</v>
       </c>
@@ -604,11 +601,11 @@
       <c r="H4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="I4" s="4">
-        <v>6383592840</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+      <c r="I4" s="3">
+        <v>6383592840</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
       <c r="A5" s="1" t="s">
         <v>14</v>
       </c>
@@ -633,11 +630,11 @@
       <c r="H5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="I5" s="4">
-        <v>6383592840</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+      <c r="I5" s="3">
+        <v>6383592840</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
       <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
@@ -662,11 +659,11 @@
       <c r="H6" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="I6" s="4">
-        <v>6383592840</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+      <c r="I6" s="3">
+        <v>6383592840</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
       <c r="A7" s="1" t="s">
         <v>16</v>
       </c>
@@ -691,11 +688,11 @@
       <c r="H7" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="I7" s="4">
-        <v>6383592840</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
+      <c r="I7" s="3">
+        <v>6383592840</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
       <c r="A8" s="1" t="s">
         <v>17</v>
       </c>
@@ -720,11 +717,11 @@
       <c r="H8" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="I8" s="4">
-        <v>6383592840</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
+      <c r="I8" s="3">
+        <v>6383592840</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
       <c r="A9" s="1" t="s">
         <v>18</v>
       </c>
@@ -749,11 +746,11 @@
       <c r="H9" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="I9" s="4">
-        <v>6383592840</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
+      <c r="I9" s="3">
+        <v>6383592840</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
       <c r="A10" s="1" t="s">
         <v>19</v>
       </c>
@@ -778,7 +775,7 @@
       <c r="H10" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="I10" s="4">
+      <c r="I10" s="3">
         <v>6383592840</v>
       </c>
     </row>
@@ -807,7 +804,7 @@
       <c r="H11" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="I11" s="4">
+      <c r="I11" s="3">
         <v>6383592840</v>
       </c>
     </row>
@@ -836,7 +833,7 @@
       <c r="H12" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="I12" s="4">
+      <c r="I12" s="3">
         <v>6383592840</v>
       </c>
     </row>
@@ -865,7 +862,7 @@
       <c r="H13" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="I13" s="4">
+      <c r="I13" s="3">
         <v>6383592840</v>
       </c>
     </row>
@@ -894,7 +891,7 @@
       <c r="H14" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="I14" s="4">
+      <c r="I14" s="3">
         <v>6383592840</v>
       </c>
     </row>
@@ -923,7 +920,7 @@
       <c r="H15" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="I15" s="4">
+      <c r="I15" s="3">
         <v>6383592840</v>
       </c>
     </row>
@@ -952,7 +949,7 @@
       <c r="H16" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="I16" s="4">
+      <c r="I16" s="3">
         <v>6383592840</v>
       </c>
     </row>
@@ -981,7 +978,7 @@
       <c r="H17" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="I17" s="4">
+      <c r="I17" s="3">
         <v>6383592840</v>
       </c>
     </row>
@@ -1010,7 +1007,7 @@
       <c r="H18" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="I18" s="4">
+      <c r="I18" s="3">
         <v>6383592840</v>
       </c>
     </row>
@@ -1039,7 +1036,7 @@
       <c r="H19" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="I19" s="4">
+      <c r="I19" s="3">
         <v>6383592840</v>
       </c>
     </row>
@@ -1068,7 +1065,7 @@
       <c r="H20" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="I20" s="4">
+      <c r="I20" s="3">
         <v>6383592840</v>
       </c>
     </row>
@@ -1097,7 +1094,7 @@
       <c r="H21" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="I21" s="4">
+      <c r="I21" s="3">
         <v>6383592840</v>
       </c>
     </row>

</xml_diff>